<commit_message>
mejoras para ejecurtar el programa sin errores de manera
</commit_message>
<xml_diff>
--- a/canciones.xlsx
+++ b/canciones.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\WEB\descargar musica\mp3-musica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD37AC8-3AF4-4E48-92C3-145FE54A692D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EE420CF-484D-4ACF-BC85-689FF7B9ACA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1910" uniqueCount="923">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1911" uniqueCount="924">
   <si>
     <t>Cancion</t>
   </si>
@@ -2791,13 +2791,16 @@
   </si>
   <si>
     <t>Esa Chica La Oreja de Van Gogh</t>
+  </si>
+  <si>
+    <t>se que bebo se que fumo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2821,6 +2824,13 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
@@ -2860,7 +2870,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2868,6 +2878,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3206,7 +3219,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="69.109375" style="3" bestFit="1" customWidth="1"/>
@@ -3217,200 +3230,76 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>884</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
-        <v>885</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>886</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>887</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>888</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>889</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>890</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>891</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
-        <v>892</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
-        <v>893</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>894</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
-        <v>895</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
-        <v>896</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
-        <v>897</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
-        <v>898</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A17" s="4" t="s">
-        <v>899</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
-        <v>901</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A20" s="4" t="s">
-        <v>902</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
-        <v>903</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A22" s="4" t="s">
-        <v>904</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A23" s="4" t="s">
-        <v>905</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A24" s="4" t="s">
-        <v>906</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A25" s="4" t="s">
-        <v>907</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A26" s="4" t="s">
-        <v>908</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A27" s="4" t="s">
-        <v>909</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A28" s="4" t="s">
-        <v>910</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A29" s="4" t="s">
-        <v>911</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A30" s="4" t="s">
-        <v>912</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A31" s="4" t="s">
-        <v>913</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A32" s="4" t="s">
-        <v>914</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A33" s="4" t="s">
-        <v>915</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A34" s="4" t="s">
-        <v>916</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A35" s="4" t="s">
-        <v>917</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A36" s="4" t="s">
-        <v>918</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A37" s="4" t="s">
-        <v>919</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A38" s="4" t="s">
-        <v>920</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A39" s="4" t="s">
-        <v>921</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" ht="15" x14ac:dyDescent="0.35">
-      <c r="A40" s="4" t="s">
-        <v>922</v>
-      </c>
+    <row r="2" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A3" s="5"/>
+    </row>
+    <row r="4" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A4" s="5"/>
+    </row>
+    <row r="5" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A5" s="5"/>
+    </row>
+    <row r="6" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A6" s="5"/>
+    </row>
+    <row r="7" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A7" s="5"/>
+    </row>
+    <row r="8" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A8" s="5"/>
+    </row>
+    <row r="9" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A9" s="5"/>
+    </row>
+    <row r="10" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A10" s="5"/>
+    </row>
+    <row r="11" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A11" s="5"/>
+    </row>
+    <row r="12" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A12" s="5"/>
+    </row>
+    <row r="13" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A13" s="5"/>
+    </row>
+    <row r="14" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A14" s="5"/>
+    </row>
+    <row r="15" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A15" s="5"/>
+    </row>
+    <row r="16" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A16" s="5"/>
+    </row>
+    <row r="17" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A17" s="5"/>
+    </row>
+    <row r="18" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A18" s="5"/>
+    </row>
+    <row r="19" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A19" s="5"/>
+    </row>
+    <row r="20" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A20" s="5"/>
+    </row>
+    <row r="21" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A21" s="5"/>
+    </row>
+    <row r="22" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A22" s="5"/>
+    </row>
+    <row r="23" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A23" s="5"/>
+    </row>
+    <row r="24" spans="1:1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A24" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3419,7 +3308,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{795EFDBD-1FC6-4DEB-8E07-5B8AF3CBC087}">
-  <dimension ref="A1:A937"/>
+  <dimension ref="A1:A976"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="69.109375" bestFit="1" customWidth="1"/>
@@ -8098,6 +7987,201 @@
     <row r="937" spans="1:1" ht="15" x14ac:dyDescent="0.35">
       <c r="A937" s="2" t="s">
         <v>399</v>
+      </c>
+    </row>
+    <row r="938" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A938" s="4" t="s">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="939" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A939" s="4" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="940" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A940" s="4" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="941" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A941" s="4" t="s">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="942" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A942" s="4" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="943" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A943" s="4" t="s">
+        <v>889</v>
+      </c>
+    </row>
+    <row r="944" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A944" s="4" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="945" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A945" s="4" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="946" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A946" s="4" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="947" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A947" s="4" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="948" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A948" s="4" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="949" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A949" s="4" t="s">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="950" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A950" s="4" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="951" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A951" s="4" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="952" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A952" s="4" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="953" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A953" s="4" t="s">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="954" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A954" s="4" t="s">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="955" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A955" s="4" t="s">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="956" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A956" s="4" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="957" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A957" s="4" t="s">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="958" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A958" s="4" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="959" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A959" s="4" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="960" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A960" s="4" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="961" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A961" s="4" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="962" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A962" s="4" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="963" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A963" s="4" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="964" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A964" s="4" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="965" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A965" s="4" t="s">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="966" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A966" s="4" t="s">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="967" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A967" s="4" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="968" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A968" s="4" t="s">
+        <v>914</v>
+      </c>
+    </row>
+    <row r="969" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A969" s="4" t="s">
+        <v>915</v>
+      </c>
+    </row>
+    <row r="970" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A970" s="4" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="971" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A971" s="4" t="s">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="972" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A972" s="4" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="973" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A973" s="4" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="974" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A974" s="4" t="s">
+        <v>920</v>
+      </c>
+    </row>
+    <row r="975" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A975" s="4" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="976" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A976" s="4" t="s">
+        <v>922</v>
       </c>
     </row>
   </sheetData>

</xml_diff>